<commit_message>
convert value in indexer filter
</commit_message>
<xml_diff>
--- a/test/res/task.xlsx
+++ b/test/res/task.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\bite\Desktop\github\xlsx-exporter\test\res\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1877A711-5BFE-48BD-9D6A-58D78B4ACC84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F93D561-9D48-44CC-A724-6B5D31344B8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-15" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="define" sheetId="9" r:id="rId1"/>
@@ -1101,7 +1101,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="739" uniqueCount="269">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="739" uniqueCount="270">
   <si>
     <t>id</t>
   </si>
@@ -1920,6 +1920,10 @@
   </si>
   <si>
     <t>[]</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>task#*.id&amp;type=MAIN</t>
     <phoneticPr fontId="8" type="noConversion"/>
   </si>
 </sst>
@@ -3950,7 +3954,7 @@
     <col min="2" max="2" width="17.875" style="9" customWidth="1"/>
     <col min="3" max="4" width="15.125" style="9" customWidth="1"/>
     <col min="5" max="5" width="26.875" style="9" customWidth="1"/>
-    <col min="6" max="6" width="8.625" style="9" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.75" style="9" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13.125" style="9" customWidth="1"/>
     <col min="8" max="8" width="23.125" style="9" customWidth="1"/>
     <col min="9" max="9" width="5" style="9" customWidth="1"/>
@@ -4184,7 +4188,7 @@
         <v>13</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>99</v>
+        <v>269</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>258</v>

</xml_diff>